<commit_message>
Report NB2 dispersion and refresh GLM outputs
Add negbin_dispersion helper so negative binomial fits report a
Pearson-chi2/df_resid ratio alongside alpha, matching the Poisson and
quasi-Poisson dispersion diagnostics. Also point the pipeline at the
db/ input directory and regenerate all GLM tables, figures, and the
results summary.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/geo_spatial_stats.xlsx
+++ b/outputs/geo_spatial_stats.xlsx
@@ -4140,7 +4140,7 @@
         <v>-0.2305058763409597</v>
       </c>
       <c r="G2" t="n">
-        <v>0.044</v>
+        <v>0.03</v>
       </c>
       <c r="H2" t="n">
         <v>4</v>
@@ -4179,7 +4179,7 @@
         <v>0.2718740988185467</v>
       </c>
       <c r="G3" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.061</v>
       </c>
       <c r="H3" t="n">
         <v>3</v>
@@ -4218,7 +4218,7 @@
         <v>0.5818847727022768</v>
       </c>
       <c r="G4" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
@@ -4257,7 +4257,7 @@
         <v>0.4100248854187086</v>
       </c>
       <c r="G5" t="n">
-        <v>0.137</v>
+        <v>0.108</v>
       </c>
       <c r="H5" t="n">
         <v>3</v>
@@ -4296,7 +4296,7 @@
         <v>0.07131373456676596</v>
       </c>
       <c r="G6" t="n">
-        <v>0.347</v>
+        <v>0.299</v>
       </c>
       <c r="H6" t="n">
         <v>3</v>
@@ -4335,7 +4335,7 @@
         <v>0.3163247183959836</v>
       </c>
       <c r="G7" t="n">
-        <v>0.121</v>
+        <v>0.102</v>
       </c>
       <c r="H7" t="n">
         <v>3</v>
@@ -4413,7 +4413,7 @@
         <v>0.8870317858091593</v>
       </c>
       <c r="G9" t="n">
-        <v>0.026</v>
+        <v>0.027</v>
       </c>
       <c r="H9" t="n">
         <v>1</v>
@@ -4452,7 +4452,7 @@
         <v>2.280217895419689</v>
       </c>
       <c r="G10" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
@@ -4491,7 +4491,7 @@
         <v>0.6524432834790829</v>
       </c>
       <c r="G11" t="n">
-        <v>0.032</v>
+        <v>0.021</v>
       </c>
       <c r="H11" t="n">
         <v>3</v>
@@ -4530,7 +4530,7 @@
         <v>0.08385414004074923</v>
       </c>
       <c r="G12" t="n">
-        <v>0.027</v>
+        <v>0.034</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -4569,7 +4569,7 @@
         <v>0.6706315369652492</v>
       </c>
       <c r="G13" t="n">
-        <v>0.013</v>
+        <v>0.018</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
@@ -4608,7 +4608,7 @@
         <v>2.188740989341055</v>
       </c>
       <c r="G14" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
@@ -4647,7 +4647,7 @@
         <v>0.5845244402044052</v>
       </c>
       <c r="G15" t="n">
-        <v>0.053</v>
+        <v>0.058</v>
       </c>
       <c r="H15" t="n">
         <v>3</v>
@@ -4686,7 +4686,7 @@
         <v>0.2752563381534771</v>
       </c>
       <c r="G16" t="n">
-        <v>0.073</v>
+        <v>0.078</v>
       </c>
       <c r="H16" t="n">
         <v>3</v>
@@ -4725,7 +4725,7 @@
         <v>0.9198146583075103</v>
       </c>
       <c r="G17" t="n">
-        <v>0.045</v>
+        <v>0.043</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
@@ -4764,7 +4764,7 @@
         <v>0.3649864242123719</v>
       </c>
       <c r="G18" t="n">
-        <v>0.079</v>
+        <v>0.093</v>
       </c>
       <c r="H18" t="n">
         <v>3</v>
@@ -4803,7 +4803,7 @@
         <v>0.4065080294215593</v>
       </c>
       <c r="G19" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="H19" t="n">
         <v>3</v>
@@ -4835,14 +4835,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LL</t>
+          <t>NS</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>0.02306950512385084</v>
       </c>
       <c r="G20" t="n">
-        <v>0.04</v>
+        <v>0.055</v>
       </c>
       <c r="H20" t="n">
         <v>3</v>
@@ -4881,7 +4881,7 @@
         <v>-0.2323766678258648</v>
       </c>
       <c r="G21" t="n">
-        <v>0.12</v>
+        <v>0.139</v>
       </c>
       <c r="H21" t="n">
         <v>2</v>
@@ -4959,7 +4959,7 @@
         <v>0.09441976601339003</v>
       </c>
       <c r="G23" t="n">
-        <v>0.344</v>
+        <v>0.371</v>
       </c>
       <c r="H23" t="n">
         <v>3</v>
@@ -4998,7 +4998,7 @@
         <v>0.6173523184517672</v>
       </c>
       <c r="G24" t="n">
-        <v>0.051</v>
+        <v>0.058</v>
       </c>
       <c r="H24" t="n">
         <v>3</v>
@@ -5037,7 +5037,7 @@
         <v>0.1317835591450095</v>
       </c>
       <c r="G25" t="n">
-        <v>0.18</v>
+        <v>0.201</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
@@ -5076,7 +5076,7 @@
         <v>0.8169046234746664</v>
       </c>
       <c r="G26" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
@@ -5115,7 +5115,7 @@
         <v>0.4063494682101423</v>
       </c>
       <c r="G27" t="n">
-        <v>0.131</v>
+        <v>0.146</v>
       </c>
       <c r="H27" t="n">
         <v>3</v>
@@ -5154,7 +5154,7 @@
         <v>-0.1373924257200849</v>
       </c>
       <c r="G28" t="n">
-        <v>0.141</v>
+        <v>0.149</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
@@ -5193,7 +5193,7 @@
         <v>-0.05162625637642825</v>
       </c>
       <c r="G29" t="n">
-        <v>0.438</v>
+        <v>0.412</v>
       </c>
       <c r="H29" t="n">
         <v>2</v>
@@ -5232,7 +5232,7 @@
         <v>-0.2717082276939747</v>
       </c>
       <c r="G30" t="n">
-        <v>0.096</v>
+        <v>0.083</v>
       </c>
       <c r="H30" t="n">
         <v>2</v>
@@ -5271,7 +5271,7 @@
         <v>0.01582102169017568</v>
       </c>
       <c r="G31" t="n">
-        <v>0.456</v>
+        <v>0.474</v>
       </c>
       <c r="H31" t="n">
         <v>3</v>
@@ -5310,7 +5310,7 @@
         <v>-0.1917384394309071</v>
       </c>
       <c r="G32" t="n">
-        <v>0.358</v>
+        <v>0.343</v>
       </c>
       <c r="H32" t="n">
         <v>2</v>
@@ -5349,7 +5349,7 @@
         <v>0.0004643340701219148</v>
       </c>
       <c r="G33" t="n">
-        <v>0.416</v>
+        <v>0.399</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
@@ -5388,7 +5388,7 @@
         <v>0.1801162261571728</v>
       </c>
       <c r="G34" t="n">
-        <v>0.329</v>
+        <v>0.312</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
@@ -5427,7 +5427,7 @@
         <v>-0.07551422182195874</v>
       </c>
       <c r="G35" t="n">
-        <v>0.435</v>
+        <v>0.443</v>
       </c>
       <c r="H35" t="n">
         <v>2</v>
@@ -5466,7 +5466,7 @@
         <v>-0.1708473183108737</v>
       </c>
       <c r="G36" t="n">
-        <v>0.333</v>
+        <v>0.332</v>
       </c>
       <c r="H36" t="n">
         <v>4</v>
@@ -5505,7 +5505,7 @@
         <v>-0.4120202658970133</v>
       </c>
       <c r="G37" t="n">
-        <v>0.117</v>
+        <v>0.107</v>
       </c>
       <c r="H37" t="n">
         <v>2</v>
@@ -5544,7 +5544,7 @@
         <v>-0.3859060287227233</v>
       </c>
       <c r="G38" t="n">
-        <v>0.165</v>
+        <v>0.166</v>
       </c>
       <c r="H38" t="n">
         <v>2</v>
@@ -5583,7 +5583,7 @@
         <v>0.7514817776341474</v>
       </c>
       <c r="G39" t="n">
-        <v>0.125</v>
+        <v>0.133</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
@@ -5622,7 +5622,7 @@
         <v>-0.9246393396318622</v>
       </c>
       <c r="G40" t="n">
-        <v>0.242</v>
+        <v>0.245</v>
       </c>
       <c r="H40" t="n">
         <v>4</v>
@@ -5661,7 +5661,7 @@
         <v>-0.3328052731892094</v>
       </c>
       <c r="G41" t="n">
-        <v>0.182</v>
+        <v>0.184</v>
       </c>
       <c r="H41" t="n">
         <v>4</v>
@@ -5700,7 +5700,7 @@
         <v>-0.2318263075084358</v>
       </c>
       <c r="G42" t="n">
-        <v>0.209</v>
+        <v>0.206</v>
       </c>
       <c r="H42" t="n">
         <v>2</v>
@@ -5739,7 +5739,7 @@
         <v>0.09397545796438352</v>
       </c>
       <c r="G43" t="n">
-        <v>0.129</v>
+        <v>0.122</v>
       </c>
       <c r="H43" t="n">
         <v>1</v>
@@ -5778,7 +5778,7 @@
         <v>0.243180236910543</v>
       </c>
       <c r="G44" t="n">
-        <v>0.244</v>
+        <v>0.246</v>
       </c>
       <c r="H44" t="n">
         <v>3</v>
@@ -5817,7 +5817,7 @@
         <v>0.09031374667393255</v>
       </c>
       <c r="G45" t="n">
-        <v>0.136</v>
+        <v>0.123</v>
       </c>
       <c r="H45" t="n">
         <v>1</v>
@@ -5856,7 +5856,7 @@
         <v>-0.1149501779287405</v>
       </c>
       <c r="G46" t="n">
-        <v>0.163</v>
+        <v>0.145</v>
       </c>
       <c r="H46" t="n">
         <v>2</v>
@@ -5895,7 +5895,7 @@
         <v>0.2962922964078399</v>
       </c>
       <c r="G47" t="n">
-        <v>0.204</v>
+        <v>0.177</v>
       </c>
       <c r="H47" t="n">
         <v>1</v>
@@ -5934,7 +5934,7 @@
         <v>0.1191836943616516</v>
       </c>
       <c r="G48" t="n">
-        <v>0.4</v>
+        <v>0.403</v>
       </c>
       <c r="H48" t="n">
         <v>3</v>
@@ -5973,7 +5973,7 @@
         <v>0.04288158655151009</v>
       </c>
       <c r="G49" t="n">
-        <v>0.307</v>
+        <v>0.304</v>
       </c>
       <c r="H49" t="n">
         <v>3</v>
@@ -6012,7 +6012,7 @@
         <v>-0.07170507666131118</v>
       </c>
       <c r="G50" t="n">
-        <v>0.182</v>
+        <v>0.173</v>
       </c>
       <c r="H50" t="n">
         <v>2</v>
@@ -6051,7 +6051,7 @@
         <v>-0.2485485170339873</v>
       </c>
       <c r="G51" t="n">
-        <v>0.062</v>
+        <v>0.051</v>
       </c>
       <c r="H51" t="n">
         <v>4</v>
@@ -6090,7 +6090,7 @@
         <v>0.1254580970642684</v>
       </c>
       <c r="G52" t="n">
-        <v>0.39</v>
+        <v>0.388</v>
       </c>
       <c r="H52" t="n">
         <v>3</v>
@@ -6168,7 +6168,7 @@
         <v>0.01736356613390224</v>
       </c>
       <c r="G54" t="n">
-        <v>0.322</v>
+        <v>0.346</v>
       </c>
       <c r="H54" t="n">
         <v>1</v>
@@ -6207,7 +6207,7 @@
         <v>-0.6791381198635622</v>
       </c>
       <c r="G55" t="n">
-        <v>0.108</v>
+        <v>0.11</v>
       </c>
       <c r="H55" t="n">
         <v>4</v>
@@ -6285,7 +6285,7 @@
         <v>-0.001282199219521999</v>
       </c>
       <c r="G57" t="n">
-        <v>0.493</v>
+        <v>0.499</v>
       </c>
       <c r="H57" t="n">
         <v>4</v>
@@ -6324,7 +6324,7 @@
         <v>-0.05761001043585837</v>
       </c>
       <c r="G58" t="n">
-        <v>0.299</v>
+        <v>0.288</v>
       </c>
       <c r="H58" t="n">
         <v>2</v>
@@ -6363,7 +6363,7 @@
         <v>-0.3125898777214013</v>
       </c>
       <c r="G59" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.093</v>
       </c>
       <c r="H59" t="n">
         <v>2</v>
@@ -6402,7 +6402,7 @@
         <v>-0.2745187963164393</v>
       </c>
       <c r="G60" t="n">
-        <v>0.133</v>
+        <v>0.13</v>
       </c>
       <c r="H60" t="n">
         <v>4</v>
@@ -6441,7 +6441,7 @@
         <v>0.03930366942545189</v>
       </c>
       <c r="G61" t="n">
-        <v>0.442</v>
+        <v>0.444</v>
       </c>
       <c r="H61" t="n">
         <v>3</v>
@@ -6480,7 +6480,7 @@
         <v>-0.2479461989232624</v>
       </c>
       <c r="G62" t="n">
-        <v>0.193</v>
+        <v>0.197</v>
       </c>
       <c r="H62" t="n">
         <v>2</v>
@@ -6519,7 +6519,7 @@
         <v>-0.2701165633050917</v>
       </c>
       <c r="G63" t="n">
-        <v>0.315</v>
+        <v>0.318</v>
       </c>
       <c r="H63" t="n">
         <v>4</v>
@@ -6558,7 +6558,7 @@
         <v>-0.03226514213756449</v>
       </c>
       <c r="G64" t="n">
-        <v>0.301</v>
+        <v>0.29</v>
       </c>
       <c r="H64" t="n">
         <v>2</v>
@@ -6597,7 +6597,7 @@
         <v>-0.08392754420419235</v>
       </c>
       <c r="G65" t="n">
-        <v>0.357</v>
+        <v>0.351</v>
       </c>
       <c r="H65" t="n">
         <v>2</v>
@@ -6636,7 +6636,7 @@
         <v>1.235858641058677</v>
       </c>
       <c r="G66" t="n">
-        <v>0.045</v>
+        <v>0.047</v>
       </c>
       <c r="H66" t="n">
         <v>1</v>
@@ -6675,7 +6675,7 @@
         <v>-0.06398360901475905</v>
       </c>
       <c r="G67" t="n">
-        <v>0.311</v>
+        <v>0.299</v>
       </c>
       <c r="H67" t="n">
         <v>4</v>
@@ -6714,7 +6714,7 @@
         <v>0.04898506920962777</v>
       </c>
       <c r="G68" t="n">
-        <v>0.466</v>
+        <v>0.452</v>
       </c>
       <c r="H68" t="n">
         <v>3</v>
@@ -6753,7 +6753,7 @@
         <v>-0.6440992691705475</v>
       </c>
       <c r="G69" t="n">
-        <v>0.025</v>
+        <v>0.032</v>
       </c>
       <c r="H69" t="n">
         <v>2</v>
@@ -6792,7 +6792,7 @@
         <v>0.003283405974879414</v>
       </c>
       <c r="G70" t="n">
-        <v>0.468</v>
+        <v>0.489</v>
       </c>
       <c r="H70" t="n">
         <v>3</v>
@@ -6831,7 +6831,7 @@
         <v>0.6268993017495619</v>
       </c>
       <c r="G71" t="n">
-        <v>0.026</v>
+        <v>0.029</v>
       </c>
       <c r="H71" t="n">
         <v>3</v>
@@ -6870,7 +6870,7 @@
         <v>-0.01013926986206695</v>
       </c>
       <c r="G72" t="n">
-        <v>0.455</v>
+        <v>0.44</v>
       </c>
       <c r="H72" t="n">
         <v>2</v>
@@ -6909,7 +6909,7 @@
         <v>-0.4543088549771213</v>
       </c>
       <c r="G73" t="n">
-        <v>0.14</v>
+        <v>0.143</v>
       </c>
       <c r="H73" t="n">
         <v>2</v>
@@ -6948,7 +6948,7 @@
         <v>-0.2473484553246046</v>
       </c>
       <c r="G74" t="n">
-        <v>0.335</v>
+        <v>0.342</v>
       </c>
       <c r="H74" t="n">
         <v>4</v>
@@ -6987,7 +6987,7 @@
         <v>0.5170621597709912</v>
       </c>
       <c r="G75" t="n">
-        <v>0.083</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H75" t="n">
         <v>3</v>
@@ -7026,7 +7026,7 @@
         <v>-0.2351708647021919</v>
       </c>
       <c r="G76" t="n">
-        <v>0.124</v>
+        <v>0.095</v>
       </c>
       <c r="H76" t="n">
         <v>4</v>
@@ -7065,7 +7065,7 @@
         <v>0.2059669377015815</v>
       </c>
       <c r="G77" t="n">
-        <v>0.16</v>
+        <v>0.159</v>
       </c>
       <c r="H77" t="n">
         <v>1</v>
@@ -7104,7 +7104,7 @@
         <v>-0.0007590950671165636</v>
       </c>
       <c r="G78" t="n">
-        <v>0.449</v>
+        <v>0.451</v>
       </c>
       <c r="H78" t="n">
         <v>4</v>
@@ -7136,14 +7136,14 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>NS</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="F79" t="n">
         <v>0.5119375351767051</v>
       </c>
       <c r="G79" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.048</v>
       </c>
       <c r="H79" t="n">
         <v>3</v>
@@ -7175,14 +7175,14 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>NS</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>0.4991670277680885</v>
       </c>
       <c r="G80" t="n">
-        <v>0.077</v>
+        <v>0.041</v>
       </c>
       <c r="H80" t="n">
         <v>3</v>
@@ -7221,7 +7221,7 @@
         <v>-0.07067713566159052</v>
       </c>
       <c r="G81" t="n">
-        <v>0.29</v>
+        <v>0.299</v>
       </c>
       <c r="H81" t="n">
         <v>2</v>
@@ -7260,7 +7260,7 @@
         <v>-1.174995686219294</v>
       </c>
       <c r="G82" t="n">
-        <v>0.246</v>
+        <v>0.207</v>
       </c>
       <c r="H82" t="n">
         <v>4</v>
@@ -7330,7 +7330,7 @@
         <v>-0.03846153846153846</v>
       </c>
       <c r="D2" t="n">
-        <v>5.38987291613109</v>
+        <v>5.5085237311644</v>
       </c>
       <c r="E2" t="n">
         <v>0.001</v>
@@ -7352,10 +7352,10 @@
         <v>-0.03846153846153846</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.3269688257832291</v>
+        <v>-0.2882315711744424</v>
       </c>
       <c r="E3" t="n">
-        <v>0.402</v>
+        <v>0.446</v>
       </c>
       <c r="F3" t="b">
         <v>0</v>
@@ -7374,10 +7374,10 @@
         <v>-0.03846153846153846</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3657902024253952</v>
+        <v>0.3272327617785755</v>
       </c>
       <c r="E4" t="n">
-        <v>0.321</v>
+        <v>0.327</v>
       </c>
       <c r="F4" t="b">
         <v>0</v>

</xml_diff>